<commit_message>
Use framed cover images in 2026-09-30 upload files
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0195ParaRQG7Bbek2o5XPZV4
</commit_message>
<xml_diff>
--- a/daily_output/Shopee_upload_MY_2026-09-30.xlsx
+++ b/daily_output/Shopee_upload_MY_2026-09-30.xlsx
@@ -13103,7 +13103,7 @@
     <t xml:space="preserve">B0CBNPSNT7</t>
   </si>
   <si>
-    <t xml:space="preserve">https://m.media-amazon.com/images/I/51r2xk2tyDL._AC_SL1202_.jpg</t>
+    <t xml:space="preserve">https://raw.githubusercontent.com/jyankel0726switch-code/ai-management-shopee/claude/admiring-bardeen-8xil2p/framed-images/B0CBNPSNT7_cover.jpg</t>
   </si>
   <si>
     <t xml:space="preserve">On</t>
@@ -13128,7 +13128,7 @@
     <t xml:space="preserve">B0CCY4Q3LG</t>
   </si>
   <si>
-    <t xml:space="preserve">https://m.media-amazon.com/images/I/51IuVjdI04L._AC_SL1079_.jpg</t>
+    <t xml:space="preserve">https://raw.githubusercontent.com/jyankel0726switch-code/ai-management-shopee/claude/admiring-bardeen-8xil2p/framed-images/B0CCY4Q3LG_cover.jpg</t>
   </si>
   <si>
     <t xml:space="preserve">https://m.media-amazon.com/images/I/51E4gk3y43L.jpg</t>
@@ -13168,7 +13168,7 @@
     <t xml:space="preserve">B0F9YHDPXQ</t>
   </si>
   <si>
-    <t xml:space="preserve">https://m.media-amazon.com/images/I/61uCyUCqgVL._AC_SL1000_.jpg</t>
+    <t xml:space="preserve">https://raw.githubusercontent.com/jyankel0726switch-code/ai-management-shopee/claude/admiring-bardeen-8xil2p/framed-images/B0F9YHDPXQ_cover.jpg</t>
   </si>
   <si>
     <t xml:space="preserve">https://m.media-amazon.com/images/I/51R1APs-boL.jpg</t>

</xml_diff>